<commit_message>
Spring menu: redesigned menu with ingredients, dietary marks, sauces and ordering
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/weeks/week-01/files/stores-and-menu.xlsx
+++ b/content/weeks/week-01/files/stores-and-menu.xlsx
@@ -701,11 +701,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -719,6 +721,16 @@
           <t>New</t>
         </is>
       </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>What's in it</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Dietary</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -727,6 +739,16 @@
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Grilled chicken, cilantro-lime rice, black beans, roasted corn, pico de gallo and Saguaro Green Sauce.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Gluten-free</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -735,6 +757,16 @@
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Grilled marinated steak, cilantro-lime rice, pinto beans, grilled onions, cotija and Chipotle Crema.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Gluten-free</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -743,6 +775,16 @@
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Pork slow-braised in green chile, brown rice, black beans, pickled red onion and queso fresco.</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Spicy, Gluten-free</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -751,6 +793,16 @@
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Roasted squash, sweet potato and peppers, brown rice, black beans and pepitas with Cilantro Lime Dressing.</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Vegetarian, Gluten-free</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -759,6 +811,16 @@
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Crispy tofu, brown rice, charred broccoli and cabbage slaw with Gochujang Glaze.</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Vegan, Spicy</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -767,6 +829,16 @@
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Romaine and mixed greens, sliced avocado, tortilla strips, corn and cherry tomatoes with Cilantro Lime Dressing.</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -775,6 +847,16 @@
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Mesquite-grilled chicken, brown rice, crunchy slaw and roasted corn with Mesquite BBQ.</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Gluten-free</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -787,6 +869,16 @@
           <t>New</t>
         </is>
       </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Charred street corn with cotija and chili-lime, black beans and cilantro-lime rice with Chipotle Crema.</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -799,6 +891,16 @@
           <t>New</t>
         </is>
       </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Grilled steak, roasted Hatch green chiles, cilantro-lime rice, pinto beans and queso fresco.</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Spicy, Gluten-free</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -811,6 +913,12 @@
           <t>New</t>
         </is>
       </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Kale and romaine, grilled chicken, parmesan and toasted seeds with a lemony Caesar dressing.</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -821,6 +929,16 @@
       <c r="B12" t="inlineStr">
         <is>
           <t>New</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Gochujang-glazed chicken, brown rice, cucumber, pickled carrots and sesame.</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Spicy</t>
         </is>
       </c>
     </row>
@@ -835,10 +953,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -847,6 +966,11 @@
           <t>Sauce</t>
         </is>
       </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -854,6 +978,11 @@
           <t>Saguaro Green Sauce</t>
         </is>
       </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Tomatillo, jalapeño and cilantro. Our signature.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -861,6 +990,11 @@
           <t>Chipotle Crema</t>
         </is>
       </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Smoky chipotle and lime, cool and creamy.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -868,6 +1002,11 @@
           <t>Cilantro Lime Dressing</t>
         </is>
       </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Bright and herby, made for greens.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -875,11 +1014,21 @@
           <t>Mesquite BBQ</t>
         </is>
       </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Sweet and smoky, with a mesquite finish.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
           <t>Gochujang Glaze</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Sweet heat from Korean chili paste.</t>
         </is>
       </c>
     </row>

</xml_diff>